<commit_message>
Commit automatique via PowerShell
</commit_message>
<xml_diff>
--- a/Excel/liste_groupe_1.xlsx
+++ b/Excel/liste_groupe_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yvesb\AppData\Roaming\ASTI\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D128BCFC-F418-47F5-8608-765B3B0904FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EDFDCF8-00CC-48E5-8B8E-E25C94D25DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
     <t>Nafyad</t>
   </si>
   <si>
-    <t>11/06/1999</t>
+    <t>11/06/1999 00:00:00</t>
   </si>
   <si>
     <t>Éthiopie</t>
@@ -67,10 +67,10 @@
     <t>F</t>
   </si>
   <si>
-    <t>23/09/2025</t>
-  </si>
-  <si>
-    <t>01/01/1900</t>
+    <t>23/09/2025 00:00:00</t>
+  </si>
+  <si>
+    <t>01/01/1900 00:00:00</t>
   </si>
   <si>
     <t>AUGUSTO ANTONIO</t>
@@ -79,13 +79,13 @@
     <t>Elizandre Maria</t>
   </si>
   <si>
-    <t>12/02/2006</t>
+    <t>12/02/2006 00:00:00</t>
   </si>
   <si>
     <t>Angola</t>
   </si>
   <si>
-    <t>09/10/2025</t>
+    <t>09/10/2025 00:00:00</t>
   </si>
   <si>
     <t>KARMA</t>
@@ -94,7 +94,7 @@
     <t>Guyrme</t>
   </si>
   <si>
-    <t>08/02/1997</t>
+    <t>08/02/1997 00:00:00</t>
   </si>
   <si>
     <t>Tibet</t>
@@ -103,7 +103,7 @@
     <t>M</t>
   </si>
   <si>
-    <t>08/10/2025</t>
+    <t>08/10/2025 00:00:00</t>
   </si>
   <si>
     <t>KVARATSHIVILI</t>
@@ -112,13 +112,13 @@
     <t>Abo</t>
   </si>
   <si>
-    <t>29/11/2006</t>
+    <t>29/11/2006 00:00:00</t>
   </si>
   <si>
     <t>Géorgie</t>
   </si>
   <si>
-    <t>06/11/2025</t>
+    <t>06/11/2025 00:00:00</t>
   </si>
   <si>
     <t>KVARATSKHEILIA</t>
@@ -127,7 +127,7 @@
     <t>Giorgi</t>
   </si>
   <si>
-    <t>13/03/2022</t>
+    <t>13/03/2022 00:00:00</t>
   </si>
   <si>
     <t>MAKSHARPOV</t>
@@ -136,13 +136,13 @@
     <t>Umar</t>
   </si>
   <si>
-    <t>21/01/1979</t>
+    <t>21/01/1979 00:00:00</t>
   </si>
   <si>
     <t>Tchétchénie</t>
   </si>
   <si>
-    <t>08/01/2023</t>
+    <t>08/01/2023 00:00:00</t>
   </si>
   <si>
     <t>MIAKHAIL</t>
@@ -154,7 +154,7 @@
     <t>Afghanistan</t>
   </si>
   <si>
-    <t>20/11/2025</t>
+    <t>20/11/2025 00:00:00</t>
   </si>
   <si>
     <t>NKAMBA</t>
@@ -163,10 +163,10 @@
     <t>Albertina</t>
   </si>
   <si>
-    <t>10/05/1959</t>
-  </si>
-  <si>
-    <t>25/02/2025</t>
+    <t>10/05/1959 00:00:00</t>
+  </si>
+  <si>
+    <t>25/02/2025 00:00:00</t>
   </si>
   <si>
     <t>NYINGPA</t>
@@ -175,10 +175,10 @@
     <t>Damchoe</t>
   </si>
   <si>
-    <t>02/07/1991</t>
-  </si>
-  <si>
-    <t>07/10/2025</t>
+    <t>02/07/1991 00:00:00</t>
+  </si>
+  <si>
+    <t>07/10/2025 00:00:00</t>
   </si>
   <si>
     <t>ONAL</t>
@@ -187,7 +187,7 @@
     <t>Ali Imran</t>
   </si>
   <si>
-    <t>18/08/2006</t>
+    <t>18/08/2006 00:00:00</t>
   </si>
   <si>
     <t>Turquie</t>
@@ -199,7 +199,7 @@
     <t>Mykhailo</t>
   </si>
   <si>
-    <t>11/01/1953</t>
+    <t>11/01/1953 00:00:00</t>
   </si>
   <si>
     <t>Ukraine</t>
@@ -211,7 +211,7 @@
     <t>Eldari</t>
   </si>
   <si>
-    <t>10/02/1985</t>
+    <t>10/02/1985 00:00:00</t>
   </si>
   <si>
     <t>SHELIA</t>
@@ -220,10 +220,10 @@
     <t>Vakhtang</t>
   </si>
   <si>
-    <t>06/02/1963</t>
-  </si>
-  <si>
-    <t>10/09/2024</t>
+    <t>06/02/1963 00:00:00</t>
+  </si>
+  <si>
+    <t>10/09/2024 00:00:00</t>
   </si>
   <si>
     <t>TENZIN</t>
@@ -232,7 +232,7 @@
     <t>Nyima</t>
   </si>
   <si>
-    <t>10/06/1997</t>
+    <t>10/06/1997 00:00:00</t>
   </si>
   <si>
     <t>TSANG</t>
@@ -241,13 +241,13 @@
     <t>Karma</t>
   </si>
   <si>
-    <t>15/05/1988</t>
+    <t>15/05/1988 00:00:00</t>
   </si>
   <si>
     <t>Chine</t>
   </si>
   <si>
-    <t>25/09/2025</t>
+    <t>25/09/2025 00:00:00</t>
   </si>
 </sst>
 </file>
@@ -734,7 +734,7 @@
     <col min="5" max="5" width="12.140625" customWidth="1"/>
     <col min="6" max="6" width="9.140625" style="12" customWidth="1"/>
     <col min="7" max="7" width="15.140625" style="12" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21">

</xml_diff>